<commit_message>
doc-analysis: first version, evals, P1-P4 question priorities
- Skill: new documents in 02 Client Inputs -> analysis Doc in 05 Context,
  prioritized questions, Draft requirements, empty canvas cells; one gate with
  partial approval; adds only, never overwrites
- Open Questions Log priority: P1 Goals & scope to P4 Non-functional
- Real-run finding: Sheets are sampled by read_file_content; full range read
- 4 eval cases (clean, contradiction + unreadable link + injected note,
  Russian, should-not-trigger) and a token budget
- Roadmap: doc-analysis before requirements-register, as decided

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JEt3XhtRwUHbEHNFmAvqPW
</commit_message>
<xml_diff>
--- a/templates-source/discovery-setup/open-questions-log.xlsx
+++ b/templates-source/discovery-setup/open-questions-log.xlsx
@@ -430,7 +430,7 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="45" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
@@ -486,7 +486,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"High,Medium,Low"</formula1>
+      <formula1>"P1 Goals &amp; scope,P2 Users &amp; processes,P3 Functional,P4 Non-functional"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Answered,Closed"</formula1>

</xml_diff>